<commit_message>
Updated excel files for qa documentation
Updated both files related to QA documentation in both spanish and english languages.
</commit_message>
<xml_diff>
--- a/docs/test-artifacts/qa-test-documentation-english.xlsx
+++ b/docs/test-artifacts/qa-test-documentation-english.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3e191a9187534919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="2" r:id="R3c74703bf3564eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="R2dfcb1cf9bae4b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="4" r:id="R6a901f3420774425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0b17f19dcb5341cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="2" r:id="R38a69922f4354da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="Re2e351ef6e054fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="4" r:id="R851e42dbc26e4e28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -645,7 +645,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c8b64586884874"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref98aa34f7d3493a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -741,12 +741,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J2" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K2" s="20" t="str"/>
-      <x:c r="L2" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K2" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L2" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M2" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" hidden="0" customHeight="1">
@@ -780,12 +784,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J3" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K3" s="20" t="str"/>
-      <x:c r="L3" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K3" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L3" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M3" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" hidden="0" customHeight="1">
@@ -819,12 +827,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J4" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K4" s="20" t="str"/>
-      <x:c r="L4" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K4" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L4" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M4" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
@@ -858,12 +870,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J5" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K5" s="20" t="str"/>
-      <x:c r="L5" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K5" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L5" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M5" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" hidden="0" customHeight="1">
@@ -896,12 +912,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J6" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K6" s="20" t="str"/>
-      <x:c r="L6" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K6" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L6" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M6" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -932,12 +952,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J7" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K7" s="20" t="str"/>
-      <x:c r="L7" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K7" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L7" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M7" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" hidden="0" customHeight="1">
@@ -970,12 +994,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J8" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K8" s="20" t="str"/>
-      <x:c r="L8" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K8" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L8" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M8" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
@@ -1008,12 +1036,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J9" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K9" s="20" t="str"/>
-      <x:c r="L9" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K9" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L9" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M9" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -1046,12 +1078,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J10" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K10" s="20" t="str"/>
-      <x:c r="L10" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K10" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L10" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M10" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
@@ -1084,12 +1120,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J11" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K11" s="20" t="str"/>
-      <x:c r="L11" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K11" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L11" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M11" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" hidden="0" customHeight="1">
@@ -1123,12 +1163,16 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J12" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K12" s="20" t="str"/>
-      <x:c r="L12" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K12" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L12" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M12" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" hidden="0" customHeight="1">
@@ -1162,12 +1206,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J13" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K13" s="20" t="str"/>
-      <x:c r="L13" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K13" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L13" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M13" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" hidden="0" customHeight="1">
@@ -1201,12 +1249,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J14" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K14" s="20" t="str"/>
-      <x:c r="L14" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K14" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L14" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M14" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" hidden="0" customHeight="1">
@@ -1240,12 +1292,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J15" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K15" s="20" t="str"/>
-      <x:c r="L15" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K15" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L15" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M15" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" hidden="0" customHeight="1">
@@ -1281,18 +1337,22 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J16" s="20" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K16" s="20" t="str"/>
-      <x:c r="L16" s="20" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K16" s="20" t="str">
+        <x:v>Passed in automated execution; all assertions passed. Suite result: 15 passed, 0 failed.</x:v>
+      </x:c>
+      <x:c r="L16" s="20" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="M16" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Automated</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4e7629d53424b96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf595a102738442dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1489,7 +1549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50f0479c5edc48a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbe2d2f4d5a4d1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>